<commit_message>
Cut CLG Mexico startup capital to USD 1.0M; add PDF outputs
- Monterrey showroom fit-out reduced to 20% of the conventional
  budget (modular display on existing structure).
- Racking, forklifts, delivery vehicles and all office equipment
  bought second-hand (~40% of new).
- Headcount halved again, 29 to 15 (CDMX 10, Monterrey 5); design,
  photography, digital ops, legal and customs brokerage outsourced.
- Startup capital falls from MXN 25.9M to MXN 18.5M (USD 1.0M).
  Year 1 now turns a profit: EBITDA 4.15M (8.4%), net 2.17M (4.4%),
  EBITDA positive from Q2. Year 3 EBITDA 47.8M, net 31.7M.
- Both deliverables also exported as PDF for easier reading.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UR8FHa3QiUDKMb81YgTRV3
</commit_message>
<xml_diff>
--- a/CLG-Mexico/CLG墨西哥项目_工作分担与执行日程表.xlsx
+++ b/CLG-Mexico/CLG墨西哥项目_工作分担与执行日程表.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>总经理 John Kim —— 一人统管两座城市（不设分公司经理层），统筹全部业务板块，并直接负责全部 IT 与数字平台开发</t>
+          <t>总经理 John Kim —— 一人统管两座城市（不设分公司经理层），统筹全部业务板块，并直接负责全部 IT 与数字平台开发；15 人精简编制，设计/摄影/代运营/法务/报关全部外包</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>总经理 · 财务总监 · 外部律所</t>
+          <t>总经理 · 财务行政主管 · 外部律所</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>总经理（直管）</t>
+          <t>总经理（直管，2人开发团队）</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理 · 外包设计团队</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>品牌总监 · 销售总监</t>
+          <t>销售总监 · 外包设计团队</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>CDMX展厅 · 蒙特雷展厅仓库 · 代理商 · 大型渠道</t>
+          <t>CDMX展厅 · 蒙特雷展厅仓库（二手设备） · 代理商 · 大型渠道</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>供应链总监 · 自有物流公司</t>
+          <t>财务行政主管（兼采购） · 自有物流公司</t>
         </is>
       </c>
     </row>
@@ -1306,12 +1306,12 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>三线差异化策略 · 地推展会 · 数字投放 · 品牌战役</t>
+          <t>三线差异化策略 · 地推展会 · 数字投放（代运营外包）</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>总经理 · 销售/品牌总监</t>
+          <t>总经理 · 销售总监</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>29人精简编制招聘 · 培训 · 绩效激励</t>
+          <t>15人精简编制招聘 · 培训 · 绩效激励</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>财务总监 · 总经理</t>
+          <t>财务行政主管 · 总经理</t>
         </is>
       </c>
     </row>
@@ -1374,8 +1374,8 @@
     <mergeCell ref="E14"/>
     <mergeCell ref="B13:F13"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>财务总监 / 供应链总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F6" s="18" t="inlineStr">
@@ -1559,12 +1559,12 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>自有品牌 Logo/VI 定稿；首批产品设计与中国确认样完成</t>
+          <t>自有品牌 Logo/VI 定稿；首批产品设计与中国确认样完成（外包设计）</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理 / 外包设计团队</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>供应链总监 / 自有物流</t>
+          <t>财务行政主管（兼采购） / 自有物流</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>总经理 / 品牌总监 / 销售总监</t>
+          <t>总经理 / 销售总监</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>总经理 / 财务总监</t>
+          <t>总经理 / 财务行政主管</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>品牌总监 / 供应链总监</t>
+          <t>总经理 / 财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>总经理 / 财务总监</t>
+          <t>总经理 / 财务行政主管</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>首年收入 4,950万比索；EBITDA 65万比索；代理商30家；活跃B2B客户180家</t>
+          <t>首年收入 4,950万比索；EBITDA 415万比索；净利润 217万比索；代理商30家；活跃B2B客户180家</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -1767,8 +1767,8 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>外部律所 / 财务总监</t>
+          <t>外部律所 / 财务行政主管</t>
         </is>
       </c>
       <c r="G5" s="22" t="n">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -2252,14 +2252,14 @@
           <t>IMPI 商标先行注册：2个品牌×全部相关尼斯类别，同周注册 .com.mx 域名与社媒账号</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>总经理（John Kim） / 律所</t>
+          <t>外包设计团队 / 律所</t>
         </is>
       </c>
       <c r="G11" s="22" t="n">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>律所 / 财务总监</t>
+          <t>律所 / 财务行政主管</t>
         </is>
       </c>
       <c r="G16" s="27" t="n">
@@ -2608,12 +2608,12 @@
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="G17" s="22" t="n">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="G18" s="27" t="n">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>IT开发组</t>
+          <t>IT开发组（2人，总经理直属）</t>
         </is>
       </c>
       <c r="G19" s="22" t="n">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>销售总监 / 财务总监</t>
+          <t>销售总监 / 财务行政主管</t>
         </is>
       </c>
       <c r="G20" s="27" t="n">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>IT开发组</t>
+          <t>IT开发组（2人，总经理直属）</t>
         </is>
       </c>
       <c r="G21" s="22" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="G22" s="27" t="n">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
-          <t>IT开发组 / 品牌总监</t>
+          <t>IT开发组 / 外包设计团队</t>
         </is>
       </c>
       <c r="G23" s="22" t="n">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>电商运营</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="G24" s="27" t="n">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
-          <t>IT开发组 / 财务</t>
+          <t>IT开发组 / 财务行政主管</t>
         </is>
       </c>
       <c r="G25" s="22" t="n">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>IT开发组</t>
+          <t>IT开发组（2人，总经理直属）</t>
         </is>
       </c>
       <c r="G26" s="27" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
-          <t>IT开发组 / 财务</t>
+          <t>IT开发组 / 财务行政主管</t>
         </is>
       </c>
       <c r="G27" s="22" t="n">
@@ -3252,17 +3252,17 @@
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>品牌定位、命名、Logo与VI视觉识别系统设计</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+          <t>品牌定位、命名、Logo与VI视觉识别系统设计（外包设计团队，不设内部编制）</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F28" s="18" t="inlineStr">
         <is>
-          <t>总经理（John Kim）</t>
+          <t>外包设计团队</t>
         </is>
       </c>
       <c r="G28" s="27" t="n">
@@ -3314,14 +3314,14 @@
           <t>首批3大品类产品设计（结构/外观/包装）与BOM确认</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E29" s="21" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>中国供应链</t>
+          <t>外包设计团队 / 中国供应链</t>
         </is>
       </c>
       <c r="G29" s="22" t="n">
@@ -3375,12 +3375,12 @@
       </c>
       <c r="E30" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="G30" s="27" t="n">
@@ -3432,14 +3432,14 @@
           <t>包装与标签本地化（西语 + NOM-050）、条码GS1申请</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E31" s="21" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>合规</t>
+          <t>外包设计团队 / 合规</t>
         </is>
       </c>
       <c r="G31" s="22" t="n">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
@@ -3550,14 +3550,14 @@
           <t>第二、三批品类扩展（累计6大品类SKU矩阵）</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>外包设计团队 / 采购</t>
         </is>
       </c>
       <c r="G33" s="22" t="n">
@@ -3609,14 +3609,14 @@
           <t>集团公司介绍手册（中/西/英）设计与印刷</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
         <is>
-          <t>总经理（John Kim）</t>
+          <t>外包设计团队 / 采购</t>
         </is>
       </c>
       <c r="G34" s="27" t="n">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>品牌总监 / 财务</t>
+          <t>外包设计团队 / 财务行政主管</t>
         </is>
       </c>
       <c r="G35" s="22" t="n">
@@ -3783,17 +3783,17 @@
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>SKU拍摄、白底图与详情页素材库（全品类）</t>
+          <t>SKU拍摄、白底图与详情页素材库（全品类，摄影外包）</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>电商运营</t>
+          <t>销售总监</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="G37" s="22" t="n">
@@ -3845,14 +3845,14 @@
           <t>展会物料、样品箱、路演PPT与投资者数据室</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F38" s="18" t="inlineStr">
         <is>
-          <t>总经理（John Kim） / 财务总监</t>
+          <t>财务行政主管 / 外包设计团队</t>
         </is>
       </c>
       <c r="G38" s="27" t="n">
@@ -4019,12 +4019,12 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>蒙特雷 3,306㎡ 仓库选址签约、货架/叉车/安防/WMS布设</t>
+          <t>蒙特雷 3,306㎡ 仓库选址签约；二手货架/二手叉车采购、安防与WMS布设</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
@@ -4319,12 +4319,12 @@
       </c>
       <c r="E46" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F46" s="18" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="G46" s="27" t="n">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="E48" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F48" s="18" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="F50" s="18" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="G50" s="27" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="F52" s="18" t="inlineStr">
         <is>
-          <t>销售总监 / 品牌总监</t>
+          <t>销售总监 / 外包设计团队</t>
         </is>
       </c>
       <c r="G52" s="27" t="n">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>市场专员</t>
+          <t>销售代表团队</t>
         </is>
       </c>
       <c r="G53" s="22" t="n">
@@ -4786,17 +4786,17 @@
       </c>
       <c r="D54" s="18" t="inlineStr">
         <is>
-          <t>B2C数字营销：Meta/Google/TikTok投放、KOL与内容运营</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>电商运营</t>
+          <t>B2C数字营销：Meta/Google/TikTok投放、KOL与内容运营（代运营外包）</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F54" s="18" t="inlineStr">
         <is>
-          <t>品牌总监</t>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="G54" s="27" t="n">
@@ -4848,14 +4848,14 @@
           <t>自有品牌上市发布会与全渠道整合营销战役</t>
         </is>
       </c>
-      <c r="E55" s="16" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="E55" s="21" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>总经理（John Kim）</t>
+          <t>外包设计团队 / 采购</t>
         </is>
       </c>
       <c r="G55" s="22" t="n">
@@ -4904,12 +4904,12 @@
       </c>
       <c r="D56" s="18" t="inlineStr">
         <is>
-          <t>组织架构定稿；墨城核心14人到岗，蒙特雷10人于第2-3月到岗（展厅开业前）</t>
+          <t>组织架构定稿；墨城核心8人到岗，蒙特雷5人于第2-3月到岗（展厅开业前）</t>
         </is>
       </c>
       <c r="E56" s="18" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F56" s="18" t="inlineStr">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="K56" s="18" t="inlineStr">
         <is>
-          <t>24人到岗</t>
+          <t>13人到岗</t>
         </is>
       </c>
       <c r="L56" s="17" t="inlineStr">
@@ -4963,17 +4963,17 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>墨城剩余5人按业务量分批到岗至满编29人；产品知识与系统培训</t>
+          <t>墨城剩余2人按业务量分批到岗至满编15人；产品知识与系统培训</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>各部门负责人</t>
+          <t>销售总监 / 蒙特雷销售主管</t>
         </is>
       </c>
       <c r="G57" s="22" t="n">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="K57" s="16" t="inlineStr">
         <is>
-          <t>满编29人 / 培训记录</t>
+          <t>满编15人 / 培训记录</t>
         </is>
       </c>
       <c r="L57" s="15" t="inlineStr">
@@ -5027,7 +5027,7 @@
       </c>
       <c r="E58" s="18" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F58" s="18" t="inlineStr">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="G59" s="22" t="n">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="E60" s="18" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F60" s="18" t="inlineStr">
@@ -5204,7 +5204,7 @@
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="E62" s="18" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F62" s="18" t="inlineStr">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="G63" s="22" t="n">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="F64" s="18" t="inlineStr">
         <is>
-          <t>财务总监 / 财务顾问</t>
+          <t>财务行政主管 / 外部财务顾问</t>
         </is>
       </c>
       <c r="G64" s="27" t="n">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
@@ -5515,7 +5515,7 @@
       <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="C8" s="38" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D8" s="40" t="n">
@@ -6194,7 +6194,7 @@
       </c>
       <c r="C9" s="44" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D9" s="46" t="n">
@@ -6269,7 +6269,7 @@
       </c>
       <c r="C10" s="38" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D10" s="40" t="n">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="C11" s="44" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D11" s="46" t="n">
@@ -6417,9 +6417,9 @@
           <t>IMPI 商标先行注册：2个品牌×全部相关尼斯类别，同周注册 .com.mx 域名与社媒账号</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D12" s="40" t="n">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="C13" s="44" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D13" s="46" t="n">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="C14" s="38" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D14" s="40" t="n">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C16" s="38" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D16" s="40" t="n">
@@ -6869,7 +6869,7 @@
       </c>
       <c r="C18" s="38" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D18" s="40" t="n">
@@ -7689,12 +7689,12 @@
       </c>
       <c r="B29" s="44" t="inlineStr">
         <is>
-          <t>品牌定位、命名、Logo与VI视觉识别系统设计</t>
-        </is>
-      </c>
-      <c r="C29" s="44" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+          <t>品牌定位、命名、Logo与VI视觉识别系统设计（外包设计团队，不设内部编制）</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D29" s="46" t="n">
@@ -7767,9 +7767,9 @@
           <t>首批3大品类产品设计（结构/外观/包装）与BOM确认</t>
         </is>
       </c>
-      <c r="C30" s="38" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D30" s="40" t="n">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="C31" s="44" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D31" s="46" t="n">
@@ -7917,9 +7917,9 @@
           <t>包装与标签本地化（西语 + NOM-050）、条码GS1申请</t>
         </is>
       </c>
-      <c r="C32" s="38" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D32" s="40" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D33" s="46" t="n">
@@ -8067,9 +8067,9 @@
           <t>第二、三批品类扩展（累计6大品类SKU矩阵）</t>
         </is>
       </c>
-      <c r="C34" s="38" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C34" s="39" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D34" s="40" t="n">
@@ -8142,9 +8142,9 @@
           <t>集团公司介绍手册（中/西/英）设计与印刷</t>
         </is>
       </c>
-      <c r="C35" s="44" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C35" s="45" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D35" s="46" t="n">
@@ -8364,12 +8364,12 @@
       </c>
       <c r="B38" s="38" t="inlineStr">
         <is>
-          <t>SKU拍摄、白底图与详情页素材库（全品类）</t>
+          <t>SKU拍摄、白底图与详情页素材库（全品类，摄影外包）</t>
         </is>
       </c>
       <c r="C38" s="38" t="inlineStr">
         <is>
-          <t>电商运营</t>
+          <t>销售总监</t>
         </is>
       </c>
       <c r="D38" s="40" t="n">
@@ -8442,9 +8442,9 @@
           <t>展会物料、样品箱、路演PPT与投资者数据室</t>
         </is>
       </c>
-      <c r="C39" s="44" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C39" s="45" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D39" s="46" t="n">
@@ -8664,12 +8664,12 @@
       </c>
       <c r="B42" s="38" t="inlineStr">
         <is>
-          <t>蒙特雷 3,306㎡ 仓库选址签约、货架/叉车/安防/WMS布设</t>
+          <t>蒙特雷 3,306㎡ 仓库选址签约；二手货架/二手叉车采购、安防与WMS布设</t>
         </is>
       </c>
       <c r="C42" s="38" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D42" s="40" t="n">
@@ -9044,7 +9044,7 @@
       </c>
       <c r="C47" s="44" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D47" s="46" t="n">
@@ -9119,7 +9119,7 @@
       </c>
       <c r="C48" s="38" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D48" s="40" t="n">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="C49" s="44" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D49" s="46" t="n">
@@ -9269,7 +9269,7 @@
       </c>
       <c r="C50" s="38" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D50" s="40" t="n">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="C52" s="38" t="inlineStr">
         <is>
-          <t>供应链总监</t>
+          <t>财务行政主管（兼采购）</t>
         </is>
       </c>
       <c r="D52" s="40" t="n">
@@ -9639,12 +9639,12 @@
       </c>
       <c r="B55" s="44" t="inlineStr">
         <is>
-          <t>B2C数字营销：Meta/Google/TikTok投放、KOL与内容运营</t>
-        </is>
-      </c>
-      <c r="C55" s="44" t="inlineStr">
-        <is>
-          <t>电商运营</t>
+          <t>B2C数字营销：Meta/Google/TikTok投放、KOL与内容运营（代运营外包）</t>
+        </is>
+      </c>
+      <c r="C55" s="45" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D55" s="46" t="n">
@@ -9717,9 +9717,9 @@
           <t>自有品牌上市发布会与全渠道整合营销战役</t>
         </is>
       </c>
-      <c r="C56" s="38" t="inlineStr">
-        <is>
-          <t>品牌总监</t>
+      <c r="C56" s="39" t="inlineStr">
+        <is>
+          <t>总经理（John Kim）</t>
         </is>
       </c>
       <c r="D56" s="40" t="n">
@@ -9789,12 +9789,12 @@
       </c>
       <c r="B57" s="44" t="inlineStr">
         <is>
-          <t>组织架构定稿；墨城核心14人到岗，蒙特雷10人于第2-3月到岗（展厅开业前）</t>
+          <t>组织架构定稿；墨城核心8人到岗，蒙特雷5人于第2-3月到岗（展厅开业前）</t>
         </is>
       </c>
       <c r="C57" s="44" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D57" s="46" t="n">
@@ -9864,12 +9864,12 @@
       </c>
       <c r="B58" s="38" t="inlineStr">
         <is>
-          <t>墨城剩余5人按业务量分批到岗至满编29人；产品知识与系统培训</t>
+          <t>墨城剩余2人按业务量分批到岗至满编15人；产品知识与系统培训</t>
         </is>
       </c>
       <c r="C58" s="38" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D58" s="40" t="n">
@@ -9944,7 +9944,7 @@
       </c>
       <c r="C59" s="44" t="inlineStr">
         <is>
-          <t>人事行政经理</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D59" s="46" t="n">
@@ -10094,7 +10094,7 @@
       </c>
       <c r="C61" s="44" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D61" s="46" t="n">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="C62" s="38" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D62" s="40" t="n">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="C63" s="44" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D63" s="46" t="n">
@@ -10469,7 +10469,7 @@
       </c>
       <c r="C66" s="38" t="inlineStr">
         <is>
-          <t>财务总监</t>
+          <t>财务行政主管</t>
         </is>
       </c>
       <c r="D66" s="40" t="n">
@@ -10553,7 +10553,7 @@
     <mergeCell ref="BB4:BE4"/>
     <mergeCell ref="F4:J4"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
@@ -10564,7 +10564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -10581,21 +10581,21 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CLG 墨西哥 · 组织与人力配置（精简至 29 人，较原方案 62 人压缩 53%）</t>
+          <t xml:space="preserve">  CLG 墨西哥 · 组织与人力配置（精简至 15 人，较原方案 62 人减少 76%）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  全负荷成本 = 税前月薪 × 1.35（IMSS社保 + INFONAVIT住房 + SAR + 年终奖15天 + 休假金 + 州工资税ISN约3%）  |  总经理一人统管两城，不设分公司经理层</t>
+          <t xml:space="preserve">  全负荷成本 = 税前月薪 × 1.35（IMSS社保 + INFONAVIT住房 + SAR + 年终奖15天 + 休假金 + 州工资税ISN约3%）  |  总经理一人统管两城；设计、摄影、代运营、法务、报关全部外包</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  墨西哥城 CDMX — 集团总部（19 人）</t>
+          <t xml:space="preserve">  墨西哥城 CDMX — 集团总部（10 人）</t>
         </is>
       </c>
     </row>
@@ -10644,7 +10644,7 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>总经理（John Kim）· 两城全面管理 + IT开发全责</t>
+          <t>总经理（John Kim）· 两城全面管理 + IT开发全责 + 定价权</t>
         </is>
       </c>
       <c r="D6" s="15" t="n">
@@ -10668,25 +10668,25 @@
     <row r="7" ht="19" customHeight="1">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>高管</t>
+          <t>销售</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>总经理助理 / 行政</t>
+          <t>销售总监</t>
         </is>
       </c>
       <c r="D7" s="17" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="52" t="n">
-        <v>22000</v>
+        <v>70000</v>
       </c>
       <c r="F7" s="52" t="n">
-        <v>22000</v>
+        <v>70000</v>
       </c>
       <c r="G7" s="52" t="n">
-        <v>29700</v>
+        <v>94500</v>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
@@ -10702,78 +10702,78 @@
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>销售总监</t>
+          <t>B2B 外销代表</t>
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="51" t="n">
-        <v>70000</v>
+        <v>18000</v>
       </c>
       <c r="F8" s="51" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="G8" s="51" t="n">
-        <v>94500</v>
+        <v>72900</v>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>第1月</t>
+          <t>第1-6月</t>
         </is>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>销售</t>
+          <t>仓储</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>B2B 外销代表</t>
+          <t>仓管 / 拣货 / 发货</t>
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E9" s="52" t="n">
-        <v>18000</v>
+        <v>11000</v>
       </c>
       <c r="F9" s="52" t="n">
-        <v>90000</v>
+        <v>22000</v>
       </c>
       <c r="G9" s="52" t="n">
-        <v>121500</v>
+        <v>29700</v>
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>第1-6月</t>
+          <t>第1-3月</t>
         </is>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>仓储</t>
+          <t>电商/IT</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>仓库主管</t>
+          <t>开发与平台工程师（总经理直属）</t>
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="51" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="F10" s="51" t="n">
-        <v>40000</v>
+        <v>90000</v>
       </c>
       <c r="G10" s="51" t="n">
-        <v>54000</v>
+        <v>121500</v>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
@@ -10784,508 +10784,365 @@
     <row r="11" ht="19" customHeight="1">
       <c r="B11" s="18" t="inlineStr">
         <is>
+          <t>财务行政</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>财务行政主管（兼采购与客服）</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="52" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F11" s="52" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G11" s="52" t="n">
+        <v>47250</v>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>第1月</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1">
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>墨西哥城合计</t>
+        </is>
+      </c>
+      <c r="C12" s="53" t="inlineStr"/>
+      <c r="D12" s="54" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="55" t="inlineStr"/>
+      <c r="F12" s="55" t="n">
+        <v>451000</v>
+      </c>
+      <c r="G12" s="55" t="n">
+        <v>608850</v>
+      </c>
+      <c r="H12" s="54" t="inlineStr"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  蒙特雷 MONTERREY — 展厅与仓库（5 人，无分公司经理层，直接向总经理汇报）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>职能</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>岗位</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>月薪(比索)</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>月薪合计</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>全负荷月成本</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>到岗时点</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="19" customHeight="1">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>销售</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>销售主管（蒙特雷负责人，直接向总经理汇报）</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="51" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F16" s="51" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G16" s="51" t="n">
+        <v>60750</v>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>第2月</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>销售</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>B2B 代表（工业/劳保方向）</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="52" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F17" s="52" t="n">
+        <v>36000</v>
+      </c>
+      <c r="G17" s="52" t="n">
+        <v>48600</v>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>第2-3月</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>销售</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>展厅顾问（兼分公司行政）</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="51" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F18" s="51" t="n">
+        <v>14000</v>
+      </c>
+      <c r="G18" s="51" t="n">
+        <v>18900</v>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>第3月</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
           <t>仓储</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>仓管 / 拣货 / 打包</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="52" t="n">
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>仓管 / 司机</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="52" t="n">
         <v>11000</v>
       </c>
-      <c r="F11" s="52" t="n">
-        <v>44000</v>
-      </c>
-      <c r="G11" s="52" t="n">
-        <v>59400</v>
-      </c>
-      <c r="H11" s="17" t="inlineStr">
-        <is>
-          <t>第1-3月</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="19" customHeight="1">
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>电商/IT</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>开发与平台工程师（总经理直属）</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" s="51" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F12" s="51" t="n">
-        <v>135000</v>
-      </c>
-      <c r="G12" s="51" t="n">
-        <v>182250</v>
-      </c>
-      <c r="H12" s="15" t="inlineStr">
-        <is>
-          <t>第1月</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="19" customHeight="1">
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>设计/品牌</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>产品与平面设计</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="52" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F13" s="52" t="n">
-        <v>35000</v>
-      </c>
-      <c r="G13" s="52" t="n">
-        <v>47250</v>
-      </c>
-      <c r="H13" s="17" t="inlineStr">
-        <is>
-          <t>第1月</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="19" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>财务/采购</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>财务负责人（兼中国采购联络）</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="51" t="n">
-        <v>40000</v>
-      </c>
-      <c r="F14" s="51" t="n">
-        <v>40000</v>
-      </c>
-      <c r="G14" s="51" t="n">
-        <v>54000</v>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
-        <is>
-          <t>第1月</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="19" customHeight="1">
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>客服</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>双语客服</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="52" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F15" s="52" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G15" s="52" t="n">
-        <v>20250</v>
-      </c>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="F19" s="52" t="n">
+        <v>11000</v>
+      </c>
+      <c r="G19" s="52" t="n">
+        <v>14850</v>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>第2月</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
-      <c r="B16" s="53" t="inlineStr">
-        <is>
-          <t>墨西哥城合计</t>
-        </is>
-      </c>
-      <c r="C16" s="53" t="inlineStr"/>
-      <c r="D16" s="54" t="n">
-        <v>19</v>
-      </c>
-      <c r="E16" s="55" t="inlineStr"/>
-      <c r="F16" s="55" t="n">
-        <v>671000</v>
-      </c>
-      <c r="G16" s="55" t="n">
-        <v>905850</v>
-      </c>
-      <c r="H16" s="54" t="inlineStr"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  蒙特雷 MONTERREY — 展厅与仓库（10 人，无分公司经理层，直接向总经理汇报）</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>职能</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>岗位</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>人数</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>月薪(比索)</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="inlineStr">
+    <row r="20" ht="19" customHeight="1">
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t>蒙特雷合计</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="inlineStr"/>
+      <c r="D20" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="55" t="inlineStr"/>
+      <c r="F20" s="55" t="n">
+        <v>106000</v>
+      </c>
+      <c r="G20" s="55" t="n">
+        <v>143100</v>
+      </c>
+      <c r="H20" s="54" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>汇总</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>编制</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>月薪合计</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>全负荷月成本</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
-        <is>
-          <t>到岗时点</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="19" customHeight="1">
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>销售</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>销售主管（蒙特雷负责人，直接向总经理汇报）</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="51" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F20" s="51" t="n">
-        <v>45000</v>
-      </c>
-      <c r="G20" s="51" t="n">
-        <v>60750</v>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>第2月</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="19" customHeight="1">
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>销售</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>B2B 代表（工业/劳保方向）</t>
-        </is>
-      </c>
-      <c r="D21" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" s="52" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F21" s="52" t="n">
-        <v>72000</v>
-      </c>
-      <c r="G21" s="52" t="n">
-        <v>97200</v>
-      </c>
-      <c r="H21" s="17" t="inlineStr">
-        <is>
-          <t>第2-3月</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="19" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>销售</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="inlineStr">
-        <is>
-          <t>展厅销售顾问</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="51" t="n">
-        <v>14000</v>
-      </c>
-      <c r="F22" s="51" t="n">
-        <v>14000</v>
-      </c>
-      <c r="G22" s="51" t="n">
-        <v>18900</v>
-      </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>第3月</t>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>年化(比索)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>仓储</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>仓管 / 司机</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="E23" s="52" t="n">
-        <v>11000</v>
-      </c>
-      <c r="F23" s="52" t="n">
-        <v>33000</v>
-      </c>
-      <c r="G23" s="52" t="n">
-        <v>44550</v>
-      </c>
-      <c r="H23" s="17" t="inlineStr">
-        <is>
-          <t>第2-3月</t>
-        </is>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>满编运行</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>墨西哥城 10 人 + 蒙特雷 5 人</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E23" s="56" t="inlineStr"/>
+      <c r="F23" s="51" t="n">
+        <v>557000</v>
+      </c>
+      <c r="G23" s="51" t="n">
+        <v>751950</v>
+      </c>
+      <c r="H23" s="51" t="n">
+        <v>9023400</v>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="B24" s="16" t="inlineStr">
-        <is>
-          <t>行政财务</t>
-        </is>
-      </c>
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>行政与会计</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="51" t="n">
-        <v>28000</v>
-      </c>
-      <c r="F24" s="51" t="n">
-        <v>28000</v>
-      </c>
-      <c r="G24" s="51" t="n">
-        <v>37800</v>
-      </c>
-      <c r="H24" s="15" t="inlineStr">
-        <is>
-          <t>第2月</t>
-        </is>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>首年实际</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>按分批到岗约75%计</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr"/>
+      <c r="E24" s="57" t="inlineStr"/>
+      <c r="F24" s="52" t="inlineStr"/>
+      <c r="G24" s="52" t="n">
+        <v>680000</v>
+      </c>
+      <c r="H24" s="52" t="n">
+        <v>6800000</v>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="B25" s="53" t="inlineStr">
-        <is>
-          <t>蒙特雷合计</t>
-        </is>
-      </c>
-      <c r="C25" s="53" t="inlineStr"/>
-      <c r="D25" s="54" t="n">
-        <v>10</v>
-      </c>
-      <c r="E25" s="55" t="inlineStr"/>
-      <c r="F25" s="55" t="n">
-        <v>192000</v>
-      </c>
-      <c r="G25" s="55" t="n">
-        <v>259200</v>
-      </c>
-      <c r="H25" s="54" t="inlineStr"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>汇总</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>编制</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr"/>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>月薪合计</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>全负荷月成本</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>年化(比索)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>满编运行</t>
-        </is>
-      </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>墨西哥城 19 人 + 蒙特雷 10 人</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>29</v>
-      </c>
-      <c r="E28" s="56" t="inlineStr"/>
-      <c r="F28" s="51" t="n">
-        <v>863000</v>
-      </c>
-      <c r="G28" s="51" t="n">
-        <v>1165050</v>
-      </c>
-      <c r="H28" s="51" t="n">
-        <v>13980600</v>
-      </c>
-    </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>首年实际</t>
-        </is>
-      </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>按分批到岗约72%计</t>
-        </is>
-      </c>
-      <c r="D29" s="17" t="inlineStr"/>
-      <c r="E29" s="57" t="inlineStr"/>
-      <c r="F29" s="52" t="inlineStr"/>
-      <c r="G29" s="52" t="n">
-        <v>1010000</v>
-      </c>
-      <c r="H29" s="52" t="n">
-        <v>10100000</v>
-      </c>
-    </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>销售提成</t>
         </is>
       </c>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>按收入 2%（4,950万比索）</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr"/>
-      <c r="E30" s="56" t="inlineStr"/>
-      <c r="F30" s="51" t="inlineStr"/>
-      <c r="G30" s="51" t="inlineStr"/>
-      <c r="H30" s="51" t="n">
+      <c r="D25" s="15" t="inlineStr"/>
+      <c r="E25" s="56" t="inlineStr"/>
+      <c r="F25" s="51" t="inlineStr"/>
+      <c r="G25" s="51" t="inlineStr"/>
+      <c r="H25" s="51" t="n">
         <v>990000</v>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="B31" s="53" t="inlineStr">
+    <row r="26" ht="19" customHeight="1">
+      <c r="B26" s="53" t="inlineStr">
         <is>
           <t>首年人力总成本</t>
         </is>
       </c>
-      <c r="C31" s="53" t="inlineStr">
-        <is>
-          <t>占首年收入 22.4%</t>
-        </is>
-      </c>
-      <c r="D31" s="54" t="inlineStr"/>
-      <c r="E31" s="58" t="inlineStr"/>
-      <c r="F31" s="55" t="inlineStr"/>
-      <c r="G31" s="55" t="inlineStr"/>
-      <c r="H31" s="55" t="n">
-        <v>11090000</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="59" t="inlineStr">
-        <is>
-          <t>较原始方案（62人）压缩 53%，年化全负荷人工由 2,678 万比索降至 1,398 万比索，节省约 1,280 万比索。取消蒙特雷分公司经理层（原月薪8万比索），改由销售主管（4.5万比索）直接向总经理汇报，单此一项年省全负荷人工约 130 万比索，并消除双城决策时延。
-薪酬仍定位于市场约120%水平（仓管 11,000 比索 vs 市场 8,400–9,700；B2B销售 18,000 底薪＋提成 vs 市场约15,000），用于吸引自带客户资源的销售人员。第二年扩编至 52 人（4城），第三年 95 人（7城），全部由经营收入承担。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35"/>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t>占首年收入 15.8%</t>
+        </is>
+      </c>
+      <c r="D26" s="54" t="inlineStr"/>
+      <c r="E26" s="58" t="inlineStr"/>
+      <c r="F26" s="55" t="inlineStr"/>
+      <c r="G26" s="55" t="inlineStr"/>
+      <c r="H26" s="55" t="n">
+        <v>7790000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="59" t="inlineStr">
+        <is>
+          <t>较原始方案（62人）减少 76%，年化全负荷人工由 2,678 万比索降至 902 万比索，节省约 1,776 万比索。取消蒙特雷分公司经理层、取消内部设计与品牌编制、财务与行政采购客服合一。
+15 人编制之所以可行：① 仓储主体在合作方寄售仓库，CLG 仅做展厅样品与周转；② 干线与末端配送由集团自有物流公司承担；③ 终端覆盖由 30→220 家代理商网络完成；④ 产品与平面设计、摄影、数字代运营、法务、报关、认证全部按项目外包，不养固定编制。15 人只负责决策、系统、大客户与渠道管理四件事。
+人均产出：第一年 330 万比索 / 人，第二年 485 万，第三年 531 万——该指标是投资人验证本编制可行性的核心 KPI。第二年扩编至 26 人（4城），第三年 48 人（7城），全部由经营收入承担。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="B14:H14"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B18:H18"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B33:H35"/>
+    <mergeCell ref="B28:H31"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -11310,14 +11167,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CLG 墨西哥 · 启动资金与资金用途（融资额 140 万美元）</t>
+          <t xml:space="preserve">  CLG 墨西哥 · 启动资金与资金用途（融资额 100 万美元）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  汇率 1 美元 = 18.50 比索  |  2亿比索货源由合作方寄售无偿供给、售出后结算，本项目无采购备货资金需求  |  第4个月起由经营收入内生</t>
+          <t xml:space="preserve">  汇率 1 美元 = 18.50 比索  |  2亿比索货源由合作方寄售无偿供给、售出后结算，无采购备货资金需求  |  装修压缩至常规方案20%，设备与车辆全部二手  |  第4个月起由经营收入内生</t>
         </is>
       </c>
     </row>
@@ -11354,18 +11211,18 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>蒙特雷展厅装修（1,653㎡，精简陈列方案）</t>
+          <t>蒙特雷展厅装修（1,653㎡，模块化陈列）</t>
         </is>
       </c>
       <c r="D5" s="51" t="n">
-        <v>3640000</v>
+        <v>728000</v>
       </c>
       <c r="E5" s="51" t="n">
-        <v>196757</v>
+        <v>39351</v>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>模块化陈列、基础灯光与夹层办公，不做重装</t>
+          <t>仅为常规装修预算的 20%；利用既有结构与照明</t>
         </is>
       </c>
     </row>
@@ -11375,18 +11232,18 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>蒙特雷仓库货架与设备</t>
+          <t>蒙特雷仓库货架与设备（全部二手）</t>
         </is>
       </c>
       <c r="D6" s="52" t="n">
-        <v>1800000</v>
+        <v>700000</v>
       </c>
       <c r="E6" s="52" t="n">
-        <v>97297</v>
+        <v>37838</v>
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>货架购置；叉车采用租赁，不占用资本</t>
+          <t>二手横梁货架、二手叉车与托盘车，约为新品 40%</t>
         </is>
       </c>
     </row>
@@ -11400,14 +11257,14 @@
         </is>
       </c>
       <c r="D7" s="51" t="n">
-        <v>900000</v>
+        <v>700000</v>
       </c>
       <c r="E7" s="51" t="n">
-        <v>48649</v>
+        <v>37838</v>
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>轻量 SaaS 方案，不自建、不上重型 ERP</t>
+          <t>轻量 SaaS，不自建、不上重型 ERP</t>
         </is>
       </c>
     </row>
@@ -11421,14 +11278,14 @@
         </is>
       </c>
       <c r="D8" s="52" t="n">
-        <v>1600000</v>
+        <v>1300000</v>
       </c>
       <c r="E8" s="52" t="n">
-        <v>86486</v>
+        <v>70270</v>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>以自有 3 人团队为主 + 定向外包</t>
+          <t>自有 2 人团队为主 + 定向外包</t>
         </is>
       </c>
     </row>
@@ -11442,14 +11299,14 @@
         </is>
       </c>
       <c r="D9" s="51" t="n">
-        <v>1200000</v>
+        <v>900000</v>
       </c>
       <c r="E9" s="51" t="n">
-        <v>64865</v>
+        <v>48649</v>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>公开发布前必须完成递交</t>
+          <t>设计按项目外包；商标须在发布前递交</t>
         </is>
       </c>
     </row>
@@ -11463,14 +11320,14 @@
         </is>
       </c>
       <c r="D10" s="52" t="n">
-        <v>600000</v>
+        <v>450000</v>
       </c>
       <c r="E10" s="52" t="n">
-        <v>32432</v>
+        <v>24324</v>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>中 / 西 / 英三语</t>
+          <t>中 / 西 / 英三语，首批小批量印刷</t>
         </is>
       </c>
     </row>
@@ -11480,18 +11337,18 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>车辆（2台配送车，租赁）+ 办公IT设备、家具、POS、监控</t>
+          <t>二手配送车 2 台 + 二手办公IT设备、家具、POS、监控</t>
         </is>
       </c>
       <c r="D11" s="51" t="n">
-        <v>1100000</v>
+        <v>500000</v>
       </c>
       <c r="E11" s="51" t="n">
-        <v>59459</v>
+        <v>27027</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>车辆租赁不购置，不占用资本</t>
+          <t>全部二手采购，不为新品付溢价</t>
         </is>
       </c>
     </row>
@@ -11501,14 +11358,14 @@
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>前 3 个月人力成本（29 人分批到岗）</t>
+          <t>前 3 个月人力成本（15 人分批到岗）</t>
         </is>
       </c>
       <c r="D12" s="52" t="n">
-        <v>2200000</v>
+        <v>1400000</v>
       </c>
       <c r="E12" s="52" t="n">
-        <v>118919</v>
+        <v>75676</v>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
@@ -11526,10 +11383,10 @@
         </is>
       </c>
       <c r="D13" s="51" t="n">
-        <v>2200000</v>
+        <v>2000000</v>
       </c>
       <c r="E13" s="51" t="n">
-        <v>118919</v>
+        <v>108108</v>
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
@@ -11575,7 +11432,7 @@
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>合规启动一次性支出</t>
+          <t>合规启动一次性支出，不可压缩</t>
         </is>
       </c>
     </row>
@@ -11610,10 +11467,10 @@
         </is>
       </c>
       <c r="D17" s="51" t="n">
-        <v>2264000</v>
+        <v>1607800</v>
       </c>
       <c r="E17" s="51" t="n">
-        <v>122378</v>
+        <v>86908</v>
       </c>
       <c r="F17" s="16" t="inlineStr">
         <is>
@@ -11629,14 +11486,14 @@
         </is>
       </c>
       <c r="D18" s="55" t="n">
-        <v>24904000</v>
+        <v>17685800</v>
       </c>
       <c r="E18" s="55" t="n">
-        <v>1346162</v>
+        <v>955989</v>
       </c>
       <c r="F18" s="53" t="inlineStr">
         <is>
-          <t>场地与信息化38% | 前3个月运营18% | 押金12% | 营运资金与备用32%</t>
+          <t>场地与信息化24% | 前3个月运营19% | 押金16% | 营运资金与备用26% | 合规8%</t>
         </is>
       </c>
     </row>
@@ -11648,14 +11505,14 @@
         </is>
       </c>
       <c r="D19" s="55" t="n">
-        <v>25900000</v>
+        <v>18500000</v>
       </c>
       <c r="E19" s="55" t="n">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="F19" s="53" t="inlineStr">
         <is>
-          <t>较原始方案 400 万美元下降 65%</t>
+          <t>较原始方案 400 万美元下降 75%</t>
         </is>
       </c>
     </row>
@@ -11751,7 +11608,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>两座新城铺设（瓜达拉哈拉、蒂华纳）、自有品牌品类扩展、团队扩编至 52 人</t>
+          <t>两座新城铺设（瓜达拉哈拉、蒂华纳）、自有品牌品类扩展、团队扩编至 26 人</t>
         </is>
       </c>
       <c r="D25" s="51" t="n">
@@ -11764,7 +11621,7 @@
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
-          <t>第二年 EBITDA 1,000 万比索支撑</t>
+          <t>第二年 EBITDA 1,920 万比索支撑</t>
         </is>
       </c>
     </row>
@@ -11776,7 +11633,7 @@
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>三座新城（莱昂、克雷塔罗、普埃布拉）、代理商扩至220家、团队95人</t>
+          <t>三座新城（莱昂、克雷塔罗、普埃布拉）、代理商扩至220家、团队48人</t>
         </is>
       </c>
       <c r="D26" s="52" t="n">
@@ -11789,7 +11646,7 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>第三年 EBITDA 3,955 万比索支撑</t>
+          <t>第三年 EBITDA 4,780 万比索支撑</t>
         </is>
       </c>
     </row>
@@ -11974,8 +11831,8 @@
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -12009,7 +11866,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  单位：百万比索  |  首年按季度、三年按年度  |  每月 5 日前由财务总监更新实际值</t>
+          <t xml:space="preserve">  单位：百万比索  |  首年按季度、三年按年度  |  每月 5 日前由财务行政主管更新实际值</t>
         </is>
       </c>
     </row>
@@ -12199,23 +12056,23 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>5.2</v>
+        <v>4.5</v>
       </c>
       <c r="D11" s="17" t="n">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>6.8</v>
+        <v>5.7</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>24.1</v>
+        <v>20.6</v>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>人力+双城租金+运营费</t>
+          <t>15人人力+双城租金+运营费</t>
         </is>
       </c>
     </row>
@@ -12226,23 +12083,23 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>-2.2</v>
+        <v>-1.5</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>-0.55</v>
+        <v>0.25</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.7</v>
+        <v>1.6</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>0.65</v>
+        <v>4.15</v>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>第三季度单季转正</t>
+          <t>第二季度单季转正；全年8.4%</t>
         </is>
       </c>
     </row>
@@ -12253,23 +12110,23 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>-2.55</v>
+        <v>-1.74</v>
       </c>
       <c r="D13" s="17" t="n">
-        <v>-0.95</v>
+        <v>-0.01</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>0.2</v>
+        <v>1.32</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>-1.1</v>
+        <v>2.17</v>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>首年小幅亏损，可结转抵税</t>
+          <t>首年即盈利，净利率4.4%</t>
         </is>
       </c>
     </row>
@@ -12286,12 +12143,12 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>启动资金</t>
+          <t>自给</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>自给</t>
+          <t>自给并再投资</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
@@ -12477,22 +12334,22 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>0.65</v>
+        <v>4.15</v>
       </c>
       <c r="D22" s="17" t="n">
-        <v>10</v>
+        <v>19.2</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>39.6</v>
+        <v>47.8</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>约125</t>
+          <t>约150</t>
         </is>
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>第三年为融资额的1.4倍</t>
+          <t>第三年为融资额的2.6倍</t>
         </is>
       </c>
       <c r="H22" s="61" t="n"/>
@@ -12505,27 +12362,27 @@
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>1.3%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>约16%</t>
+          <t>约19%</t>
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>固定成本经营杠杆</t>
+          <t>精简编制 + 固定成本经营杠杆</t>
         </is>
       </c>
       <c r="H23" s="61" t="n"/>
@@ -12537,22 +12394,22 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>-1.1</v>
+        <v>2.17</v>
       </c>
       <c r="D24" s="17" t="n">
-        <v>5.4</v>
+        <v>12.2</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>24.8</v>
+        <v>31.7</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>约86</t>
+          <t>约101</t>
         </is>
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>三年累计29.1</t>
+          <t>首年即盈利；三年累计46.1</t>
         </is>
       </c>
       <c r="H24" s="61" t="n"/>
@@ -12743,17 +12600,17 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>2 / 29</t>
+          <t>2 / 15</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>4 / 52</t>
+          <t>4 / 26</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>7 / 95</t>
+          <t>7 / 48</t>
         </is>
       </c>
       <c r="F31" s="15" t="inlineStr">
@@ -12763,7 +12620,7 @@
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>轻资产扩张纪律</t>
+          <t>极致轻资产扩张纪律</t>
         </is>
       </c>
       <c r="H31" s="61" t="n"/>
@@ -12775,13 +12632,13 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1.71</v>
+        <v>3.3</v>
       </c>
       <c r="D32" s="17" t="n">
-        <v>2.42</v>
+        <v>4.85</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>2.68</v>
+        <v>5.31</v>
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
@@ -12790,7 +12647,7 @@
       </c>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>29人编制的效率验证</t>
+          <t>15人编制可行性的核心验证指标</t>
         </is>
       </c>
       <c r="H32" s="61" t="n"/>
@@ -12798,7 +12655,7 @@
     <row r="34">
       <c r="B34" s="62" t="inlineStr">
         <is>
-          <t>五年纳斯达克路径（保守口径）：第五年营收约4,220万美元、净利率约11%（净利约464万美元）、自有品牌占比50%以上，税前利润远超纳斯达克全球市场收益标准所需的100万美元；按1.8倍 EV/Revenue 或22倍 P/E 测算，隐含企业价值 7,500万–1亿美元，相当于对首年140万美元启动资金 50–70 倍回报。三项前提：自第一年起四大/PCAOB审计、离岸控股架构、符合SOX的内控与常设资料室。</t>
+          <t>五年纳斯达克路径（保守口径）：第五年营收约4,220万美元、净利率约13%（净利约548万美元）、自有品牌占比50%以上，税前利润远超纳斯达克全球市场收益标准所需的100万美元；按1.8倍 EV/Revenue 或22倍 P/E 测算，隐含企业价值 7,500万–1.2亿美元，相当于对首年100万美元启动资金 75–120 倍回报。三项前提：自第一年起四大/PCAOB审计、离岸控股架构、符合SOX的内控与常设资料室。</t>
         </is>
       </c>
     </row>
@@ -12826,7 +12683,7 @@
     <mergeCell ref="G31:H31"/>
     <mergeCell ref="G22:H22"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Double CLG Mexico revenue plan; credit John Kim as author
- Revenue restated at 60% of the internal projection, twice the
  prior version: Y1 99.0M, Y2 252.0M, Y3 510.0M MXN.
- Gross margin lowered to 47/45/44% to reflect the channel discount
  needed for the higher volume and the shift to normal replenishment
  in year 3, once the consignment stock is 81% drawn down.
- Headcount 15 to 18; the incremental coverage comes from the agent
  network (60/180/440) rather than in-house staff.
- Startup capital MXN 21.3M (USD 1.15M); the increase over the prior
  USD 1.0M is receivables float and first-quarter payroll only.
- Year 1 EBITDA 15.88M (16.0%) and net profit 10.28M (10.4%);
  Y3 EBITDA 96.9M, 4.6x the raise.
- John Kim set as author on both files, on the plan cover and in the
  document properties.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UR8FHa3QiUDKMb81YgTRV3
</commit_message>
<xml_diff>
--- a/CLG-Mexico/CLG墨西哥项目_工作分担与执行日程表.xlsx
+++ b/CLG-Mexico/CLG墨西哥项目_工作分担与执行日程表.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>总经理 John Kim —— 一人统管两座城市（不设分公司经理层），统筹全部业务板块，并直接负责全部 IT 与数字平台开发；15 人精简编制，设计/摄影/代运营/法务/报关全部外包</t>
+          <t>总经理 John Kim —— 一人统管两座城市（不设分公司经理层），统筹全部业务板块，并直接负责全部 IT 与数字平台开发；18 人精简编制，设计/摄影/代运营/法务/报关全部外包</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>15人精简编制招聘 · 培训 · 绩效激励</t>
+          <t>18人精简编制招聘 · 培训 · 绩效激励</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>首年收入 4,950万比索；EBITDA 415万比索；净利润 217万比索；代理商30家；活跃B2B客户180家</t>
+          <t>首年收入 9,900万比索；EBITDA 1,588万比索；净利润 1,028万比索；代理商60家；活跃B2B客户360家</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="D42" s="18" t="inlineStr">
         <is>
-          <t>两城 180 家活跃 B2B 客户开发与首单转化</t>
+          <t>两城 360 家活跃 B2B 客户开发与首单转化</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="K42" s="18" t="inlineStr">
         <is>
-          <t>180个活跃账户</t>
+          <t>360个活跃账户</t>
         </is>
       </c>
       <c r="L42" s="17" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>代理商体系招募：首年30家签约（含独家条款与最低采购量）</t>
+          <t>代理商体系招募：首年60家签约（含独家条款与最低采购量）</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="K43" s="16" t="inlineStr">
         <is>
-          <t>30份代理协议</t>
+          <t>60份代理协议</t>
         </is>
       </c>
       <c r="L43" s="15" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="D56" s="18" t="inlineStr">
         <is>
-          <t>组织架构定稿；墨城核心8人到岗，蒙特雷5人于第2-3月到岗（展厅开业前）</t>
+          <t>组织架构定稿；墨城核心9人到岗，蒙特雷6人于第2-3月到岗（展厅开业前）</t>
         </is>
       </c>
       <c r="E56" s="18" t="inlineStr">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="K56" s="18" t="inlineStr">
         <is>
-          <t>13人到岗</t>
+          <t>15人到岗</t>
         </is>
       </c>
       <c r="L56" s="17" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>墨城剩余2人按业务量分批到岗至满编15人；产品知识与系统培训</t>
+          <t>墨城剩余3人按业务量分批到岗至满编18人；产品知识与系统培训</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="K57" s="16" t="inlineStr">
         <is>
-          <t>满编15人 / 培训记录</t>
+          <t>满编18人 / 培训记录</t>
         </is>
       </c>
       <c r="L57" s="15" t="inlineStr">
@@ -8739,7 +8739,7 @@
       </c>
       <c r="B43" s="44" t="inlineStr">
         <is>
-          <t>两城 180 家活跃 B2B 客户开发与首单转化</t>
+          <t>两城 360 家活跃 B2B 客户开发与首单转化</t>
         </is>
       </c>
       <c r="C43" s="44" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B44" s="38" t="inlineStr">
         <is>
-          <t>代理商体系招募：首年30家签约（含独家条款与最低采购量）</t>
+          <t>代理商体系招募：首年60家签约（含独家条款与最低采购量）</t>
         </is>
       </c>
       <c r="C44" s="38" t="inlineStr">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B57" s="44" t="inlineStr">
         <is>
-          <t>组织架构定稿；墨城核心8人到岗，蒙特雷5人于第2-3月到岗（展厅开业前）</t>
+          <t>组织架构定稿；墨城核心9人到岗，蒙特雷6人于第2-3月到岗（展厅开业前）</t>
         </is>
       </c>
       <c r="C57" s="44" t="inlineStr">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="B58" s="38" t="inlineStr">
         <is>
-          <t>墨城剩余2人按业务量分批到岗至满编15人；产品知识与系统培训</t>
+          <t>墨城剩余3人按业务量分批到岗至满编18人；产品知识与系统培训</t>
         </is>
       </c>
       <c r="C58" s="38" t="inlineStr">
@@ -10581,7 +10581,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CLG 墨西哥 · 组织与人力配置（精简至 15 人，较原方案 62 人减少 76%）</t>
+          <t xml:space="preserve">  CLG 墨西哥 · 组织与人力配置（18 人，较原方案 62 人减少 71%）</t>
         </is>
       </c>
     </row>
@@ -10595,7 +10595,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  墨西哥城 CDMX — 集团总部（10 人）</t>
+          <t xml:space="preserve">  墨西哥城 CDMX — 集团总部（12 人）</t>
         </is>
       </c>
     </row>
@@ -10706,16 +10706,16 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8" s="51" t="n">
         <v>18000</v>
       </c>
       <c r="F8" s="51" t="n">
-        <v>54000</v>
+        <v>72000</v>
       </c>
       <c r="G8" s="51" t="n">
-        <v>72900</v>
+        <v>97200</v>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
@@ -10735,16 +10735,16 @@
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" s="52" t="n">
         <v>11000</v>
       </c>
       <c r="F9" s="52" t="n">
-        <v>22000</v>
+        <v>33000</v>
       </c>
       <c r="G9" s="52" t="n">
-        <v>29700</v>
+        <v>44550</v>
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
@@ -10818,21 +10818,21 @@
       </c>
       <c r="C12" s="53" t="inlineStr"/>
       <c r="D12" s="54" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" s="55" t="inlineStr"/>
       <c r="F12" s="55" t="n">
-        <v>451000</v>
+        <v>480000</v>
       </c>
       <c r="G12" s="55" t="n">
-        <v>608850</v>
+        <v>648000</v>
       </c>
       <c r="H12" s="54" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  蒙特雷 MONTERREY — 展厅与仓库（5 人，无分公司经理层，直接向总经理汇报）</t>
+          <t xml:space="preserve">  蒙特雷 MONTERREY — 展厅与仓库（6 人，无分公司经理层，直接向总经理汇报）</t>
         </is>
       </c>
     </row>
@@ -10914,16 +10914,16 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" s="52" t="n">
         <v>18000</v>
       </c>
       <c r="F17" s="52" t="n">
-        <v>36000</v>
+        <v>54000</v>
       </c>
       <c r="G17" s="52" t="n">
-        <v>48600</v>
+        <v>72900</v>
       </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
@@ -10997,14 +10997,14 @@
       </c>
       <c r="C20" s="53" t="inlineStr"/>
       <c r="D20" s="54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" s="55" t="inlineStr"/>
       <c r="F20" s="55" t="n">
-        <v>106000</v>
+        <v>124000</v>
       </c>
       <c r="G20" s="55" t="n">
-        <v>143100</v>
+        <v>167400</v>
       </c>
       <c r="H20" s="54" t="inlineStr"/>
     </row>
@@ -11045,21 +11045,21 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>墨西哥城 10 人 + 蒙特雷 5 人</t>
+          <t>墨西哥城 12 人 + 蒙特雷 6 人</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E23" s="56" t="inlineStr"/>
       <c r="F23" s="51" t="n">
-        <v>557000</v>
+        <v>604000</v>
       </c>
       <c r="G23" s="51" t="n">
-        <v>751950</v>
+        <v>815400</v>
       </c>
       <c r="H23" s="51" t="n">
-        <v>9023400</v>
+        <v>9784800</v>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
@@ -11077,10 +11077,10 @@
       <c r="E24" s="57" t="inlineStr"/>
       <c r="F24" s="52" t="inlineStr"/>
       <c r="G24" s="52" t="n">
-        <v>680000</v>
+        <v>730000</v>
       </c>
       <c r="H24" s="52" t="n">
-        <v>6800000</v>
+        <v>7300000</v>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>按收入 2%（4,950万比索）</t>
+          <t>按收入 2%（9,900万比索）</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr"/>
@@ -11099,7 +11099,7 @@
       <c r="F25" s="51" t="inlineStr"/>
       <c r="G25" s="51" t="inlineStr"/>
       <c r="H25" s="51" t="n">
-        <v>990000</v>
+        <v>1980000</v>
       </c>
     </row>
     <row r="26" ht="19" customHeight="1">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="C26" s="53" t="inlineStr">
         <is>
-          <t>占首年收入 15.8%</t>
+          <t>仅占首年收入 9.4%</t>
         </is>
       </c>
       <c r="D26" s="54" t="inlineStr"/>
@@ -11118,15 +11118,15 @@
       <c r="F26" s="55" t="inlineStr"/>
       <c r="G26" s="55" t="inlineStr"/>
       <c r="H26" s="55" t="n">
-        <v>7790000</v>
+        <v>9280000</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="59" t="inlineStr">
         <is>
-          <t>较原始方案（62人）减少 76%，年化全负荷人工由 2,678 万比索降至 902 万比索，节省约 1,776 万比索。取消蒙特雷分公司经理层、取消内部设计与品牌编制、财务与行政采购客服合一。
-15 人编制之所以可行：① 仓储主体在合作方寄售仓库，CLG 仅做展厅样品与周转；② 干线与末端配送由集团自有物流公司承担；③ 终端覆盖由 30→220 家代理商网络完成；④ 产品与平面设计、摄影、数字代运营、法务、报关、认证全部按项目外包，不养固定编制。15 人只负责决策、系统、大客户与渠道管理四件事。
-人均产出：第一年 330 万比索 / 人，第二年 485 万，第三年 531 万——该指标是投资人验证本编制可行性的核心 KPI。第二年扩编至 26 人（4城），第三年 48 人（7城），全部由经营收入承担。</t>
+          <t>较原始方案（62人）减少 71%，年化全负荷人工 978 万比索。取消蒙特雷分公司经理层、取消内部设计与品牌编制、财务与行政采购客服合一。收入较上一版翻倍仅增加 3 名一线人员（销售 2、仓储 1）。
+18 人编制之所以可行：① 仓储主体在合作方寄售仓库，CLG 仅做展厅样品与周转；② 干线与末端配送由集团自有物流公司承担；③ 终端覆盖由 60→440 家代理商网络完成，增量收入主要由代理商而非自建团队实现；④ 产品与平面设计、摄影、数字代运营、法务、报关、认证全部按项目外包，不养固定编制。18 人只负责决策、系统、大客户与渠道管理四件事。
+人均产出：第一年 550 万比索 / 人，第二年 663 万，第三年 708 万——该指标是投资人验证本编制可行性的核心 KPI。第二年扩编至 38 人（4城），第三年 72 人（7城），全部由经营收入承担。</t>
         </is>
       </c>
     </row>
@@ -11167,7 +11167,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CLG 墨西哥 · 启动资金与资金用途（融资额 100 万美元）</t>
+          <t xml:space="preserve">  CLG 墨西哥 · 启动资金与资金用途（融资额 115 万美元）</t>
         </is>
       </c>
     </row>
@@ -11358,14 +11358,14 @@
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>前 3 个月人力成本（15 人分批到岗）</t>
+          <t>前 3 个月人力成本（18 人分批到岗）</t>
         </is>
       </c>
       <c r="D12" s="52" t="n">
-        <v>1400000</v>
+        <v>1700000</v>
       </c>
       <c r="E12" s="52" t="n">
-        <v>75676</v>
+        <v>91892</v>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
@@ -11383,10 +11383,10 @@
         </is>
       </c>
       <c r="D13" s="51" t="n">
-        <v>2000000</v>
+        <v>2300000</v>
       </c>
       <c r="E13" s="51" t="n">
-        <v>108108</v>
+        <v>124324</v>
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
@@ -11446,14 +11446,14 @@
         </is>
       </c>
       <c r="D16" s="52" t="n">
-        <v>3000000</v>
+        <v>5000000</v>
       </c>
       <c r="E16" s="52" t="n">
-        <v>162162</v>
+        <v>270270</v>
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>仅为账期垫付，占收入 6%</t>
+          <t>仅为账期垫付，占收入 5%</t>
         </is>
       </c>
     </row>
@@ -11467,10 +11467,10 @@
         </is>
       </c>
       <c r="D17" s="51" t="n">
-        <v>1607800</v>
+        <v>1867800</v>
       </c>
       <c r="E17" s="51" t="n">
-        <v>86908</v>
+        <v>100962</v>
       </c>
       <c r="F17" s="16" t="inlineStr">
         <is>
@@ -11486,14 +11486,14 @@
         </is>
       </c>
       <c r="D18" s="55" t="n">
-        <v>17685800</v>
+        <v>20545800</v>
       </c>
       <c r="E18" s="55" t="n">
-        <v>955989</v>
+        <v>1110584</v>
       </c>
       <c r="F18" s="53" t="inlineStr">
         <is>
-          <t>场地与信息化24% | 前3个月运营19% | 押金16% | 营运资金与备用26% | 合规8%</t>
+          <t>场地与信息化21% | 前3个月运营19% | 押金14% | 营运资金与备用33% | 合规7%</t>
         </is>
       </c>
     </row>
@@ -11505,14 +11505,14 @@
         </is>
       </c>
       <c r="D19" s="55" t="n">
-        <v>18500000</v>
+        <v>21300000</v>
       </c>
       <c r="E19" s="55" t="n">
-        <v>1000000</v>
+        <v>1150000</v>
       </c>
       <c r="F19" s="53" t="inlineStr">
         <is>
-          <t>较原始方案 400 万美元下降 75%</t>
+          <t>较原始方案 400 万美元下降 71%</t>
         </is>
       </c>
     </row>
@@ -11562,7 +11562,7 @@
         </is>
       </c>
       <c r="D23" s="51" t="n">
-        <v>1800000</v>
+        <v>3500000</v>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
@@ -11583,11 +11583,11 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>SKU 品类扩展、市场推广加码、代理商体系铺开、第三城前置筹备、平台 V2.0</t>
+          <t>SKU 品类扩展、市场推广加码、代理商体系铺开（60家）、第三城前置筹备、平台 V2.0</t>
         </is>
       </c>
       <c r="D24" s="52" t="n">
-        <v>5500000</v>
+        <v>9000000</v>
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>首年内生再投资合计约 730 万比索</t>
+          <t>首年内生再投资合计约 1,250 万比索</t>
         </is>
       </c>
     </row>
@@ -11608,11 +11608,11 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>两座新城铺设（瓜达拉哈拉、蒂华纳）、自有品牌品类扩展、团队扩编至 26 人</t>
+          <t>两座新城铺设（瓜达拉哈拉、蒂华纳）、代理商扩至180家、团队扩编至 38 人</t>
         </is>
       </c>
       <c r="D25" s="51" t="n">
-        <v>12000000</v>
+        <v>25000000</v>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
@@ -11621,7 +11621,7 @@
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
-          <t>第二年 EBITDA 1,920 万比索支撑</t>
+          <t>第二年 EBITDA 4,380 万比索支撑</t>
         </is>
       </c>
     </row>
@@ -11633,11 +11633,11 @@
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>三座新城（莱昂、克雷塔罗、普埃布拉）、代理商扩至220家、团队48人</t>
+          <t>三座新城（莱昂、克雷塔罗、普埃布拉）、代理商扩至440家、团队72人</t>
         </is>
       </c>
       <c r="D26" s="52" t="n">
-        <v>25000000</v>
+        <v>50000000</v>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
@@ -11646,7 +11646,7 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>第三年 EBITDA 4,780 万比索支撑</t>
+          <t>第三年 EBITDA 9,690 万比索支撑</t>
         </is>
       </c>
     </row>
@@ -11820,7 +11820,7 @@
       </c>
       <c r="F35" s="53" t="inlineStr">
         <is>
-          <t>占首年收入12.8%；第二年约9.2%，第三年约6.3%</t>
+          <t>仅占首年收入6.4%；第二年约4.6%，第三年约3.3%</t>
         </is>
       </c>
     </row>
@@ -11859,14 +11859,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CLG 墨西哥 · 销售计划与投资人监控看板（保守口径：按内部测算值 30% 计列）</t>
+          <t xml:space="preserve">  CLG 墨西哥 · 销售计划与投资人监控看板（按内部测算值 60% 计列）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  单位：百万比索  |  首年按季度、三年按年度  |  每月 5 日前由财务行政主管更新实际值</t>
+          <t xml:space="preserve">  单位：百万比索  |  首年按季度、三年按年度  |  编制人：总经理 John Kim  |  每月 5 日前由财务行政主管更新实际值</t>
         </is>
       </c>
     </row>
@@ -11921,23 +11921,23 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>10.5</v>
+        <v>21</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>49.5</v>
+        <v>99</v>
       </c>
       <c r="H6" s="16" t="inlineStr">
         <is>
-          <t>按内部测算值30%保守计列</t>
+          <t>按内部测算值60%计列</t>
         </is>
       </c>
     </row>
@@ -11948,19 +11948,19 @@
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>4.8</v>
+        <v>9.6</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>8.4</v>
+        <v>16.8</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>11.2</v>
+        <v>22.4</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>15.2</v>
+        <v>30.4</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>39.6</v>
+        <v>79.2</v>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
@@ -11975,19 +11975,19 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>1.1</v>
+        <v>2.3</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>1.5</v>
+        <v>3.1</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>5.4</v>
+        <v>10.8</v>
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
@@ -12002,19 +12002,19 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>4.5</v>
+        <v>9</v>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
@@ -12025,27 +12025,27 @@
     <row r="10" ht="19" customHeight="1">
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>毛利润（毛利率50%）</t>
+          <t>毛利润（毛利率47%）</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>3</v>
+        <v>5.64</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>5.25</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>7</v>
+        <v>13.16</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>9.5</v>
+        <v>17.86</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>24.75</v>
+        <v>46.53</v>
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>寄售货源成本优势</t>
+          <t>放量让价，毛利率由50%降至47%</t>
         </is>
       </c>
     </row>
@@ -12056,23 +12056,23 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>4.5</v>
+        <v>6.4</v>
       </c>
       <c r="D11" s="17" t="n">
-        <v>5</v>
+        <v>7.3</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>5.4</v>
+        <v>8</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>5.7</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>20.6</v>
+        <v>30.65</v>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>15人人力+双城租金+运营费</t>
+          <t>18人人力+双城租金+运营费</t>
         </is>
       </c>
     </row>
@@ -12083,23 +12083,23 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>-1.5</v>
+        <v>-0.76</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.25</v>
+        <v>2.57</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>1.6</v>
+        <v>5.16</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>3.8</v>
+        <v>8.91</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>4.15</v>
+        <v>15.88</v>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>第二季度单季转正；全年8.4%</t>
+          <t>第二季度单季转正；全年16.0%</t>
         </is>
       </c>
     </row>
@@ -12110,23 +12110,23 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>-1.74</v>
+        <v>-1.03</v>
       </c>
       <c r="D13" s="17" t="n">
-        <v>-0.01</v>
+        <v>1.9</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>1.32</v>
+        <v>3.39</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>2.6</v>
+        <v>6.02</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>2.17</v>
+        <v>10.28</v>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>首年即盈利，净利率4.4%</t>
+          <t>首年净利率10.4%</t>
         </is>
       </c>
     </row>
@@ -12241,22 +12241,22 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>49.5</v>
+        <v>99</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>126</v>
+        <v>252</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>255</v>
+        <v>510</v>
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>约780</t>
+          <t>约1,560</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>保守口径，超额部分为纯上行</t>
+          <t>保留40%安全边际，超额为纯上行</t>
         </is>
       </c>
       <c r="H19" s="61" t="n"/>
@@ -12302,27 +12302,27 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>47.0%</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>45.0%</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>约45%</t>
+          <t>约43%</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>寄售优势递减、品牌毛利接棒</t>
+          <t>放量让价 + 第三年转常规补货</t>
         </is>
       </c>
       <c r="H21" s="61" t="n"/>
@@ -12334,22 +12334,22 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>4.15</v>
+        <v>15.88</v>
       </c>
       <c r="D22" s="17" t="n">
-        <v>19.2</v>
+        <v>43.8</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>47.8</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>约150</t>
+          <t>约300</t>
         </is>
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>第三年为融资额的2.6倍</t>
+          <t>第三年为融资额的4.6倍</t>
         </is>
       </c>
       <c r="H22" s="61" t="n"/>
@@ -12362,17 +12362,17 @@
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
@@ -12394,22 +12394,22 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>2.17</v>
+        <v>10.28</v>
       </c>
       <c r="D24" s="17" t="n">
-        <v>12.2</v>
+        <v>29.1</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>31.7</v>
+        <v>65.3</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>约101</t>
+          <t>约203</t>
         </is>
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>首年即盈利；三年累计46.1</t>
+          <t>首年即盈利；三年累计104.7</t>
         </is>
       </c>
       <c r="H24" s="61" t="n"/>
@@ -12480,17 +12480,17 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F27" s="15" t="inlineStr">
@@ -12500,7 +12500,7 @@
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
-          <t>对合作方的累计结算额</t>
+          <t>第三年起转入常规补货</t>
         </is>
       </c>
       <c r="H27" s="61" t="n"/>
@@ -12512,13 +12512,13 @@
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>180</v>
+        <v>360</v>
       </c>
       <c r="D28" s="17" t="n">
-        <v>520</v>
+        <v>1040</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>1150</v>
+        <v>2300</v>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
@@ -12539,13 +12539,13 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D29" s="15" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>220</v>
+        <v>440</v>
       </c>
       <c r="F29" s="15" t="inlineStr">
         <is>
@@ -12554,7 +12554,7 @@
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>价格优势消失后的持久资产</t>
+          <t>增量收入的主要实现渠道</t>
         </is>
       </c>
       <c r="H29" s="61" t="n"/>
@@ -12600,17 +12600,17 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>2 / 15</t>
+          <t>2 / 18</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>4 / 26</t>
+          <t>4 / 38</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>7 / 48</t>
+          <t>7 / 72</t>
         </is>
       </c>
       <c r="F31" s="15" t="inlineStr">
@@ -12632,13 +12632,13 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>3.3</v>
+        <v>5.5</v>
       </c>
       <c r="D32" s="17" t="n">
-        <v>4.85</v>
+        <v>6.63</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>5.31</v>
+        <v>7.08</v>
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>15人编制可行性的核心验证指标</t>
+          <t>18人编制可行性的核心验证指标</t>
         </is>
       </c>
       <c r="H32" s="61" t="n"/>
@@ -12655,7 +12655,7 @@
     <row r="34">
       <c r="B34" s="62" t="inlineStr">
         <is>
-          <t>五年纳斯达克路径（保守口径）：第五年营收约4,220万美元、净利率约13%（净利约548万美元）、自有品牌占比50%以上，税前利润远超纳斯达克全球市场收益标准所需的100万美元；按1.8倍 EV/Revenue 或22倍 P/E 测算，隐含企业价值 7,500万–1.2亿美元，相当于对首年100万美元启动资金 75–120 倍回报。三项前提：自第一年起四大/PCAOB审计、离岸控股架构、符合SOX的内控与常设资料室。</t>
+          <t>五年纳斯达克路径：第五年营收约8,430万美元、净利率约13%（净利约1,096万美元）、自有品牌占比50%以上，税前利润远超纳斯达克全球市场收益标准所需的100万美元；按1.8倍 EV/Revenue 或22倍 P/E 测算，隐含企业价值 1.5亿–2.4亿美元，相当于对首年115万美元启动资金 130–210 倍回报。三项前提：自第一年起四大/PCAOB审计、离岸控股架构、符合SOX的内控与常设资料室。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore FY1 quarterly P&L; finish workbook visuals
- The quarterly profit-and-loss table was lost in the cover redesign,
  leaving only its chart. Restored to page 2 alongside the annual
  summary. Dropped the return-on-investment table that replaced it:
  its figures already appear in the highlights and the Nasdaq path.
- Workbook: landscape CLG banner on the overview sheet in the cover's
  design language; use-of-funds donut added to the budget sheet and
  the margin and own-brand charts to the KPI sheet.
- Wording aligned across both files (总投资金额, 启动投资), sheet ⑥
  renamed, and the project row now states the 60% revenue basis.
- Audited both deliverables for stale figures and terminology; clean.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UR8FHa3QiUDKMb81YgTRV3
</commit_message>
<xml_diff>
--- a/CLG-Mexico/CLG墨西哥项目_工作分担与执行日程表.xlsx
+++ b/CLG-Mexico/CLG墨西哥项目_工作分担与执行日程表.xlsx
@@ -12,14 +12,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ 任务分解 WBS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="④ 甘特图 Gantt" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑤ 人力配置" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑥ 启动资金与租金" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑥ 总投资额与租金" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑦ 销售与KPI目标" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'① 项目总览'!$A$1:$G$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'① 项目总览'!$A$1:$G$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'③ 任务分解 WBS'!$A$4:$M$65</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'③ 任务分解 WBS'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'④ 甘特图 Gantt'!$4:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'⑥ 总投资额与租金'!$A$1:$F$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'⑦ 销售与KPI目标'!$A$1:$H$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,17 +40,6 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -94,6 +85,17 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -178,16 +180,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0B2545"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF13315C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF2F4F7"/>
       </patternFill>
     </fill>
@@ -198,12 +190,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF13315C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B2545"/>
       </patternFill>
     </fill>
     <fill>
@@ -405,48 +407,54 @@
   </cellStyleXfs>
   <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -454,11 +462,20 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -475,43 +492,42 @@
     <xf numFmtId="9" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -524,27 +540,13 @@
     <xf numFmtId="165" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -556,10 +558,10 @@
     <xf numFmtId="3" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -704,10 +706,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6191250" cy="2762250"/>
+    <ext cx="14287500" cy="2257425"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -729,10 +731,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>45</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3000375" cy="2324100"/>
+    <ext cx="8572500" cy="3819525"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -752,12 +754,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>45</row>
+      <row>61</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3000375" cy="2038350"/>
+    <ext cx="4095750" cy="3171825"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -765,6 +767,116 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>61</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4095750" cy="2790825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7239000" cy="4067175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4000500" cy="3133725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4000500" cy="2514600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1067,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="B14:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1079,438 +1191,449 @@
     <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLG 墨西哥 · 工作分解与执行日程表</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Work Breakdown Structure &amp; Master Schedule  |  周期：2026年10月 – 2027年9月  |  编制人：总经理 John Kim  |  机密文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+    <row r="1" ht="20" customHeight="1"/>
+    <row r="2" ht="20" customHeight="1"/>
+    <row r="3" ht="20" customHeight="1"/>
+    <row r="4" ht="20" customHeight="1"/>
+    <row r="5" ht="20" customHeight="1"/>
+    <row r="6" ht="20" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1"/>
+    <row r="8" ht="20" customHeight="1"/>
+    <row r="9" ht="20" customHeight="1"/>
+    <row r="10" ht="20" customHeight="1"/>
+    <row r="11" ht="20" customHeight="1"/>
+    <row r="12" ht="20" customHeight="1"/>
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>项目名称</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>CLG 墨西哥双城启动暨全国批发网络建设项目（保守测算版）</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>CLG 墨西哥双城启动暨全国批发网络建设项目（收入按内部测算值 60% 计列）</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>启动城市</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>墨西哥城（CDMX，集团总部+800㎡展厅；货源存于合作方仓库，不自建大仓） / 蒙特雷（MTY，1,653㎡展厅+3,306㎡仓库）</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>项目总负责</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>总经理 John Kim —— 一人统管两座城市（不设分公司经理层），统筹全部业务板块，并直接负责全部 IT 与数字平台开发；18 人精简编制，设计/摄影/代运营/法务/报关全部外包</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>核心任务数</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>61 项工作包 / 九大工作流，分三个阶段推进</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="B8" s="3" t="inlineStr">
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>第一阶段</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>0–2个月（2026.10–2026.11）：寄售协议签署、三大平台开发、自有品牌打样、蒙特雷展厅与仓库落成</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>第二阶段</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>3–6个月（2026.12–2027.03）：渠道铺开、代理商体系、自有品牌量产上市；第4个月起经营现金流自给</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="B10" s="3" t="inlineStr">
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>第三阶段</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>7–12个月（2027.04–2027.09）：大型渠道准入、第三城前置、扩张支出全部由经营收入内生</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>使用说明</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>「③ 任务分解」为主控表，可按阶段／工作流／负责人筛选；「④ 甘特图」按周着色；「状态」与「进度%」为周例会更新字段；「⑤⑦」为人力与业绩台账</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  九大工作流 (Workstreams)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>流</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>工作流名称</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>核心内容</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>主责</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="8" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>公司治理与合规</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>寄售协议 / 实体 / 税务 / CFDI / IMMEX / NOM / 商标</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>总经理 · 财务行政主管 · 外部律所</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="11" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>IT与数字平台</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>官网 · B2B平台 · 品牌独立站 · ERP/WMS</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>总经理（直管，2人开发团队）</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="8" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>自有品牌开发</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>定位 · Logo/VI · 产品设计 · 打样 · 量产</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>总经理 · 外包设计团队</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="11" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>品牌物料与商务文件</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>公司手册 · 产品图册价目表 · 代理商合同</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>销售总监 · 外包设计团队</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="8" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>网点与渠道</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>CDMX展厅 · 蒙特雷展厅仓库（二手设备） · 代理商 · 大型渠道</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>总经理 · 销售总监 · MTY销售主管</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="11" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>供应链与库存</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>寄售SKU对接 · 美墨陆路通道 · 中国补货 · 清关</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>财务行政主管（兼采购） · 自有物流公司</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="8" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>市场营销</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>三线差异化策略 · 地推展会 · 数字投放（代运营外包）</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>总经理 · 销售总监</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="11" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>人力与组织</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>18人精简编制招聘 · 培训 · 绩效激励</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>财务行政主管</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="8" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>财务与资本运作</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>预算 · 授信 · 内生再投资 · IFRS审计 · 上市路径</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>财务行政主管 · 总经理</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="14" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  双城起步与三年全国铺设</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="15" customHeight="1"/>
-    <row r="28" ht="15" customHeight="1"/>
-    <row r="29" ht="15" customHeight="1"/>
-    <row r="30" ht="15" customHeight="1"/>
-    <row r="31" ht="15" customHeight="1"/>
-    <row r="32" ht="15" customHeight="1"/>
-    <row r="33" ht="15" customHeight="1"/>
-    <row r="34" ht="15" customHeight="1"/>
-    <row r="35" ht="15" customHeight="1"/>
-    <row r="36" ht="15" customHeight="1"/>
-    <row r="37" ht="15" customHeight="1"/>
-    <row r="38" ht="15" customHeight="1"/>
-    <row r="39" ht="15" customHeight="1"/>
-    <row r="40" ht="15" customHeight="1"/>
-    <row r="41" ht="15" customHeight="1"/>
-    <row r="42" ht="15" customHeight="1"/>
-    <row r="43" ht="15" customHeight="1"/>
-    <row r="45" ht="22" customHeight="1">
-      <c r="B45" s="14" t="inlineStr">
+    <row r="36" ht="18" customHeight="1"/>
+    <row r="37" ht="18" customHeight="1"/>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42" ht="18" customHeight="1"/>
+    <row r="43" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1"/>
+    <row r="46" ht="18" customHeight="1"/>
+    <row r="47" ht="18" customHeight="1"/>
+    <row r="48" ht="18" customHeight="1"/>
+    <row r="49" ht="18" customHeight="1"/>
+    <row r="50" ht="18" customHeight="1"/>
+    <row r="51" ht="18" customHeight="1"/>
+    <row r="52" ht="18" customHeight="1"/>
+    <row r="53" ht="18" customHeight="1"/>
+    <row r="54" ht="18" customHeight="1"/>
+    <row r="55" ht="18" customHeight="1"/>
+    <row r="56" ht="18" customHeight="1"/>
+    <row r="57" ht="18" customHeight="1"/>
+    <row r="58" ht="18" customHeight="1"/>
+    <row r="59" ht="18" customHeight="1">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  收入结构演进与首年分季度损益</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1"/>
-    <row r="47" ht="15" customHeight="1"/>
-    <row r="48" ht="15" customHeight="1"/>
-    <row r="49" ht="15" customHeight="1"/>
-    <row r="50" ht="15" customHeight="1"/>
-    <row r="51" ht="15" customHeight="1"/>
-    <row r="52" ht="15" customHeight="1"/>
-    <row r="53" ht="15" customHeight="1"/>
-    <row r="54" ht="15" customHeight="1"/>
-    <row r="55" ht="15" customHeight="1"/>
-    <row r="56" ht="15" customHeight="1"/>
-    <row r="57" ht="15" customHeight="1"/>
-    <row r="58" ht="15" customHeight="1"/>
-    <row r="59" ht="15" customHeight="1"/>
-    <row r="60" ht="15" customHeight="1"/>
-    <row r="61" ht="15" customHeight="1"/>
-    <row r="62">
-      <c r="B62" t="inlineStr">
+    <row r="62" ht="18" customHeight="1"/>
+    <row r="63" ht="18" customHeight="1"/>
+    <row r="64" ht="18" customHeight="1"/>
+    <row r="65" ht="18" customHeight="1"/>
+    <row r="66" ht="18" customHeight="1"/>
+    <row r="67" ht="18" customHeight="1"/>
+    <row r="68" ht="18" customHeight="1"/>
+    <row r="69" ht="18" customHeight="1"/>
+    <row r="70" ht="18" customHeight="1"/>
+    <row r="71" ht="18" customHeight="1"/>
+    <row r="72" ht="18" customHeight="1"/>
+    <row r="73" ht="18" customHeight="1"/>
+    <row r="74" ht="18" customHeight="1"/>
+    <row r="75" ht="18" customHeight="1"/>
+    <row r="76" ht="18" customHeight="1"/>
+    <row r="77" ht="18" customHeight="1"/>
+    <row r="78" ht="18" customHeight="1"/>
+    <row r="79" ht="18" customHeight="1"/>
+    <row r="80" ht="18" customHeight="1"/>
+    <row r="81" ht="18" customHeight="1">
+      <c r="B81" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="E14"/>
-    <mergeCell ref="B13:F13"/>
+  <mergeCells count="12">
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B61:F61"/>
+    <mergeCell ref="E24"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="B35:F35"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -1537,14 +1660,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLG 墨西哥 · 关键里程碑与验收标准</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  Milestones &amp; Acceptance Criteria  |  未达成里程碑须在周例会提出补救方案</t>
         </is>
@@ -1806,7 +1929,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>经营现金流自给：第4个月起不再动用启动资金，扩张支出改由经营收入承担</t>
+          <t>经营现金流自给：第4个月起不再动用启动投资，扩张支出改由经营收入承担</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
@@ -1936,14 +2059,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLG 墨西哥 · 任务分解主控表 (WBS Master)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  共 61 项工作包  |  负责人到岗即生效  |  周例会更新「状态」与「进度%」</t>
         </is>
@@ -5728,14 +5851,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLG 墨西哥 · 12个月执行甘特图 (52周)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  2026年10月 第1周  →  2027年9月 第52周   ▌深蓝=第一阶段 0-2月   ▌青色=第二阶段 3-6月   ▌金色=第三阶段 7-12月</t>
         </is>
@@ -10718,21 +10841,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLG 墨西哥 · 组织与人力配置（18 人，较原方案 62 人减少 71%）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  全负荷成本 = 税前月薪 × 1.35（IMSS社保 + INFONAVIT住房 + SAR + 年终奖15天 + 休假金 + 州工资税ISN约3%）  |  总经理一人统管两城；设计、摄影、代运营、法务、报关全部外包</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  墨西哥城 CDMX — 集团总部（12 人）</t>
         </is>
@@ -10969,7 +11092,7 @@
       <c r="H12" s="54" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  蒙特雷 MONTERREY — 展厅与仓库（6 人，无分公司经理层，直接向总经理汇报）</t>
         </is>
@@ -11148,29 +11271,29 @@
       <c r="H20" s="54" t="inlineStr"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr"/>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>编制</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>月薪合计</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>全负荷月成本</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>年化(比索)</t>
         </is>
@@ -11291,7 +11414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -11304,14 +11427,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLG 墨西哥 · 总投资金额与资金用途（约 115 万美元）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  汇率 1 美元 = 18.50 比索  |  货源由合作方寄售无偿供给、售出后结算，无采购备货资金需求  |  装修压缩至常规方案20%，设备与车辆全部二手  |  编制人：总经理 John Kim</t>
         </is>
@@ -11656,7 +11779,7 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  第 4 个月起的内生再投资计划（不再需要追加股权融资）</t>
         </is>
@@ -11790,7 +11913,7 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  双城租金模型</t>
         </is>
@@ -11963,15 +12086,55 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  总投资金额用途构成</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42" ht="18" customHeight="1"/>
+    <row r="43" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1"/>
+    <row r="46" ht="18" customHeight="1"/>
+    <row r="47" ht="18" customHeight="1"/>
+    <row r="48" ht="18" customHeight="1"/>
+    <row r="49" ht="18" customHeight="1"/>
+    <row r="50" ht="18" customHeight="1"/>
+    <row r="51" ht="18" customHeight="1"/>
+    <row r="52" ht="18" customHeight="1"/>
+    <row r="53" ht="18" customHeight="1"/>
+    <row r="54" ht="18" customHeight="1"/>
+    <row r="55" ht="18" customHeight="1"/>
+    <row r="56" ht="18" customHeight="1"/>
+    <row r="57" ht="18" customHeight="1"/>
+    <row r="58" ht="18" customHeight="1"/>
+    <row r="59" ht="18" customHeight="1"/>
+    <row r="60" ht="18" customHeight="1"/>
+    <row r="61" ht="18" customHeight="1"/>
+    <row r="62" ht="18" customHeight="1">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B21:F21"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B37:F37"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11981,7 +12144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -11996,21 +12159,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLG 墨西哥 · 销售计划与投资人监控看板（按内部测算值 60% 计列）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  单位：百万比索  |  首年按季度、三年按年度  |  编制人：总经理 John Kim  |  每月 5 日前由财务行政主管更新实际值</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  首年分季度销售与损益计划</t>
         </is>
@@ -12334,7 +12497,7 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  三年扩张与投资人 KPI 看板</t>
         </is>
@@ -12799,8 +12962,41 @@
       </c>
     </row>
     <row r="35"/>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  利润率演进与自有品牌占比</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42" ht="18" customHeight="1"/>
+    <row r="43" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1"/>
+    <row r="46" ht="18" customHeight="1"/>
+    <row r="47" ht="18" customHeight="1"/>
+    <row r="48" ht="18" customHeight="1"/>
+    <row r="49" ht="18" customHeight="1"/>
+    <row r="50" ht="18" customHeight="1"/>
+    <row r="51" ht="18" customHeight="1"/>
+    <row r="52" ht="18" customHeight="1"/>
+    <row r="53" ht="18" customHeight="1"/>
+    <row r="54" ht="18" customHeight="1"/>
+    <row r="55" ht="18" customHeight="1"/>
+    <row r="56" ht="18" customHeight="1"/>
+    <row r="57" ht="18" customHeight="1">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="G23:H23"/>
@@ -12812,6 +13008,7 @@
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="G30:H30"/>
+    <mergeCell ref="B37:F37"/>
     <mergeCell ref="G26:H26"/>
     <mergeCell ref="G29:H29"/>
     <mergeCell ref="G20:H20"/>
@@ -12824,5 +13021,6 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>